<commit_message>
simulafoot_nlg: penalty-variant -- condition mandatory gabarit == "penalty" sur les 15 phrases BUT/PENALTY
Source (classeur, colonne Condition, 15 cellules : seules differences verifiees feuille par
feuille), CHECKSUM.txt mis a jour, scenarios.yml reconverti (checksum verifie ; la
reconversion de l'etat precedent etait identique ; seules ces 15 phrases changent, d'une
condition). Sans elle, ces phrases sans condition etaient toujours candidates et essayees
avant SURNOM/DEFAUT. Tests : 15 conditions presentes, aucune autre phrase ne conditionne sur
gabarit, aucun candidat PENALTY pour un but ordinaire (6 gabarits dont None), 15 pour un
penalty ; DEFAUT inchange. La base locale se met a jour par reset-seed --yes puis import-seed.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/simulafoot_nlg/data/seed_source/banque_de_phrases_simulafoot.xlsx
+++ b/simulafoot_nlg/data/seed_source/banque_de_phrases_simulafoot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Phrases" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Dictionnaires de slots" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Preferred moves disponibles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phrases" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionnaires de slots" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preferred moves disponibles" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1801,6 +1801,11 @@
           <t>{joueur} s'avance sereinement, prend une profonde inspiration et envoie le penalty en pleine lucarne, imparable !</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F35" t="n">
         <v>1</v>
       </c>
@@ -1831,6 +1836,11 @@
           <t>{joueur} ne change pas sa course, frappe fort et au centre : le gardien s'est jeté, mais le ballon rentre en plein milieu !</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
@@ -1861,6 +1871,11 @@
           <t>Sang-froid total : {joueur} attend que le gardien de {adversaire} se couche et pousse tranquillement le ballon de l'autre côté !</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F37" t="n">
         <v>1</v>
       </c>
@@ -1891,6 +1906,11 @@
           <t>{joueur} tente une Panenka totalement décomplexée, le ballon finit tout doucement au fond sous les huées du public adverse !</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F38" t="n">
         <v>1</v>
       </c>
@@ -1921,6 +1941,11 @@
           <t>{joueur} frappe une fusée dans l'angle, le gardien part du bon côté mais ne peut rien faire face à tant de puissance !</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
@@ -1951,6 +1976,11 @@
           <t>Après un temps d'arrêt interminable, {joueur} déroute le gardien d'un enchaînement de petits pas et loge le ballon à l'opposé !</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F40" t="n">
         <v>1</v>
       </c>
@@ -1981,6 +2011,11 @@
           <t>{joueur} ne laisse paraître aucune émotion, frappe sèchement et bas dans le coin, le gardien est resté cloué sur place !</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F41" t="n">
         <v>1</v>
       </c>
@@ -2011,6 +2046,11 @@
           <t>Le stade retient son souffle, {joueur} prend son élan et catapulte le ballon au ras du poteau, personne n'y peut rien !</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F42" t="n">
         <v>1</v>
       </c>
@@ -2041,6 +2081,11 @@
           <t>{joueur} place son penalty avec une précision chirurgicale dans la lucarne opposée, le gardien de {adversaire} n'a même pas bougé !</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F43" t="n">
         <v>1</v>
       </c>
@@ -2071,6 +2116,11 @@
           <t>D'un tir croisé et puissant, {joueur} transforme sans trembler ce penalty décisif !</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
@@ -2101,6 +2151,11 @@
           <t>{joueur} feinte sa course d'un temps suspendu et surprend totalement le gardien, qui s'écroule du mauvais côté !</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F45" t="n">
         <v>1</v>
       </c>
@@ -2131,6 +2186,11 @@
           <t>{joueur} frappe fort et haut, le ballon claque sous la barre avant de finir au fond des filets !</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F46" t="n">
         <v>1</v>
       </c>
@@ -2161,6 +2221,11 @@
           <t>Malgré la pression, {joueur} garde son sang-froid et ajuste parfaitement sa frappe dans la lucarne !</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F47" t="n">
         <v>1</v>
       </c>
@@ -2191,6 +2256,11 @@
           <t>{joueur} ne tremble pas d'un poil et transforme ce penalty capital comme si de rien n'était !</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
+        </is>
+      </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
@@ -2219,6 +2289,11 @@
       <c r="D49" t="inlineStr">
         <is>
           <t>{joueur} choisit son côté avec assurance, frappe puissamment et voit le ballon se loger au fond, sans appel !</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>gabarit == "penalty"</t>
         </is>
       </c>
       <c r="F49" t="n">

</xml_diff>

<commit_message>
banque CARTON_ROUGE : 5, 11, 19, 22, 30 -- condition secondaire a la place de Aggression >= 70/75 seule (57 % -> 14-29 %)
5 intervention a retardement : Aggression >= 70 & Tackling <= 55 ; 11 contact anodin / melee : Aggression >= 75 & Determination
>= 80 ; 19 tacle desespere : Aggression >= 70 & minute >= 60 ; 22 apres un but litigieux : Aggression >= 75 & Teamwork >= 80 ;
30 tac au tac : Aggression >= 75 & Decisions <= 60. Source : classeur banque_de_phrases_simulafoot.xlsx (CHECKSUM.txt mis a jour),
scenarios.yml regenere par convert-commentary (diff = les 5 conditions ajoutees).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/simulafoot_nlg/data/seed_source/banque_de_phrases_simulafoot.xlsx
+++ b/simulafoot_nlg/data/seed_source/banque_de_phrases_simulafoot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phrases" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionnaires de slots" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preferred moves disponibles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Phrases" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dictionnaires de slots" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Preferred moves disponibles" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Aggression &gt;= 70</t>
+          <t>Aggression &gt;= 70 et Tackling &lt;= 55</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Aggression &gt;= 75</t>
+          <t>Aggression &gt;= 75 et Determination &gt;= 80</t>
         </is>
       </c>
       <c r="F144" t="n">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Aggression &gt;= 70</t>
+          <t>Aggression &gt;= 70 et minute &gt;= 60</t>
         </is>
       </c>
       <c r="F152" t="n">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Aggression &gt;= 75</t>
+          <t>Aggression &gt;= 75 et Teamwork &gt;= 80</t>
         </is>
       </c>
       <c r="F155" t="n">
@@ -5323,7 +5323,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Aggression &gt;= 75</t>
+          <t>Aggression &gt;= 75 et Decisions &lt;= 60</t>
         </is>
       </c>
       <c r="F163" t="n">

</xml_diff>